<commit_message>
feat(ui): add responsive layout foundation
- add valid viewport initialization with bounded fallback
- add Desktop, CompactLandscape, and provisional MobileLandscape modes
- add debounced viewport resize handling
- add reusable layout calculations through UILayoutCoordinator
- reflow existing BattleHUD panels without rebuilding the HUD
- preserve targeting and battle state during viewport changes
- retain existing panel names and input-blocking behavior

UAT:
- bootstrap passed
- Desktop layout passed
- Desktop and CompactLandscape breakpoint switching passed
- targeting state survived viewport resizing
- no duplicate HUD or runtime regression observed

Pending:
- MobileLandscape visual validation
- final approved panel placement
- existing action-panel and TurnOrder overlap
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Build_Plan.xlsx
+++ b/docs/CTRBLXAI_Build_Plan.xlsx
@@ -27,6 +27,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 — Validation Matrix" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 Roblox Platform" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 Implementation Plan" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 Slice Ownership" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 — Service Boundaries'!$A$4:$G$16</definedName>
@@ -479,26 +480,6 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="350" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{9C948352-E8DA-483A-8010-207117E2A654}">
-  <we:reference id="WA200010611" version="1.0.10036.0" store="en-us" storeType="OMEX"/>
-  <we:alternateReferences/>
-  <we:properties>
-    <we:property name="Office.AutoShowTaskpaneWithDocument" value="true"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -7870,7 +7851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -9029,6 +9010,1741 @@
           <t>Not designed yet. Single-player server instances assumed for now.</t>
         </is>
       </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>SLICE NUMBERING NOTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>The vertical slices above (1-10) are Build Plan implementation stages from the v5 architecture handoff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>The Development Roadmap owns the project-facing 7-slice structure (Slices 1-7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Mapping: Roadmap Slice 1 ≈ BP stages 1-3, Roadmap Slice 4 ≈ BP stages 4+6, Roadmap Slice 5 ≈ BP stage 7, Roadmap Slice 6 ≈ BP stages 5+8+9+10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>The Development Roadmap slice numbering is authoritative for current status and order.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E82"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>SLICE MODULE OWNERSHIP AND INTEGRATION POLICY</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr"/>
+      <c r="C1" t="inlineStr"/>
+      <c r="D1" t="inlineStr"/>
+      <c r="E1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FOUR MODULE CLASSIFICATIONS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Write Access</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Later Slice Rules</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Primarily owned by one slice</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Owning slice: normal. After completion: protected.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Consume through public APIs only</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Protected Completed</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Belongs to a completed slice</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Read-only for later slices</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>No rewrite for convenience, style, cleanup, refactoring</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Shared Integration</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Multiple systems meet here</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Requires: exact purpose, smallest diff, approval, regression, checkpoint</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>No unrelated cleanup. Ownership does not transfer.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Content/Config Authority</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CTRBLXAI.db, definitions, templates</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Designer agent owns. Game Rules is authoritative.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Presentation must not change gameplay values</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MODULE OWNERSHIP TABLE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BattleCoordinator.lua</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ServerScriptService/Game</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Slice 1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Protected Completed</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Battle lifecycle, CT/RT, turns</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>UnitSchema.lua</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ServerScriptService/Game</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Slice 1 + Slice 4 extension</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Shared Integration</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Slice 4 added equipment/persistent fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GameConstants.lua</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/CTRBLXAI/Shared</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Slice 1 + extensions</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Shared Integration</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>All slices may add constants; no removal/change of existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TargetingService.lua</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ServerScriptService/Game</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Slice 2</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Protected Completed</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Movement, range, targeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TileDefinitions.lua</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/CTRBLXAI/Shared</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Slice 2</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Protected Completed</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Terrain types</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CommandService.lua</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ServerScriptService/Game</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Slice 3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Protected Completed</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Command validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CombatResolver.lua</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ServerScriptService/Game</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Slice 3</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Protected Completed</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Damage/healing math</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>StatusService.lua</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ServerScriptService/Game</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Slice 3</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Protected Completed</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Status lifecycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BattleVisualBroadcaster.lua</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ServerScriptService/Game</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Slice 3</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Shared Integration</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Server→client events; payload additions need approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SaveService.lua</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ServerScriptService/Game</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>DataStore persistence</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PersistentStateService.lua</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ServerScriptService/Game</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Persistent HP/MP, recovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>InventoryService.lua</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ServerScriptService/Game</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Item storage, management</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EquipmentService.lua</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ServerScriptService/Game</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Equip/unequip, stat rebuild</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ItemGenerator.lua</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ServerScriptService/Game</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Procedural item creation</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>RegionGenerator.lua</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ServerScriptService</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Slice 5</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Region ownership grid</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TemplateViewer.server.lua</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ServerScriptService</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Slice 5</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Template/map viewer (prototype)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BattleHUD.lua</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/CTRBLXAI/UI</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Battle UI composition</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Theme.lua</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/CTRBLXAI/UI</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Colors, typography, spacing</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>UIConstants.lua</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/CTRBLXAI/UI</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>UI constants</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>UIFormatting.lua</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/CTRBLXAI/UI</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Display formatting</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>UIComponents.lua</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/CTRBLXAI/UI</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Reusable UI components</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>UILayoutCoordinator.lua</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/CTRBLXAI/UI</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Responsive layout</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>UIController.client.lua</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>StarterPlayerScripts/UI</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Client UI controller</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>UnitInspectorPanel.client.lua</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>StarterPlayerScripts</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Slice-Owned</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Unit inspection panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>CameraController.lua</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>StarterPlayerScripts</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Slice-Owned (presentation)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Camera + input routing; changes need camera regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Main.server.lua</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ServerScriptService</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Shared</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Shared Integration</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Battle orchestration, AI; all slices hook in</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BattleEvents.lua</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/CTRBLXAI/Remotes</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Shared</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Shared Integration</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>RemoteEvents consumed by multiple slices</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>BattleVisualClient.client.lua</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>StarterPlayerScripts</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Shared</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Shared Integration</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Mixed: rendering + input + state. Slice 7 reads only; hooks need approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>default.project.json</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Root</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Shared</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Shared Integration</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Rojo config; structural changes only</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Registry.lua</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/Content</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Content/Config Authority</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Generated from DB — Auditor Class C checks staleness</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SkillData.lua</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/Content</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Content/Config Authority</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>107 skills from DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AugmentData.lua</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/Content</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Content/Config Authority</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>102 augments from DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>DoctrineData.lua</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/Content</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Content/Config Authority</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>32 doctrines from DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>WeaponData.lua</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/Content</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Content/Config Authority</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Weapon archetypes from DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>BonusData.lua</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/Content</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Content/Config Authority</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Bonus attributes from DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>T01_FrontlinePressure.lua</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ReplicatedStorage/CTRBLXAI/Templates</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Content/Config Authority</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Template definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>PROTECTED COMPLETED BEHAVIOR</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>After a slice is completed, its behavior is frozen. Later slices must not:</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>- Rewrite internals for convenience, style, or cleanup</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>- Create duplicate formula implementations</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>- Create parallel state caches</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>- Infer authoritative values from visual events</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Backward-compatible additions may be approved via the compatibility process.</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>DEPENDENCY DIRECTION</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Authoritative rules/content → gameplay services → shared events/payloads → functional controllers → presentation views</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Forbidden: combat→UI, map gen→visual layout, save→UI state, targeting→highlight appearance, formulas→presentation assets</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>MIXED-SCRIPT POLICY</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BattleVisualClient.client.lua</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Shared Integration</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Mixed responsibility (rendering + input + state). Future prompts must not use as general location for new logic.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Main.server.lua</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Shared Integration</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Mixed responsibility (orchestration + AI + hooks). Modifications need exact purpose + smallest diff.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>BattleEvents.lua</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Shared Integration</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Multiple slices consume. Additions need approval; no removal of existing events.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>default.project.json</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Shared Integration</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Structural only. Do not add arbitrary paths.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>OUT-OF-BATTLE OWNERSHIP</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Functional Owner</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Visual Owner</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Roster/Inventory/Equipment</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Slice 4 owns transactions; Slice 7 displays and emits intent</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Loadouts/Deployment</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Slice 4 owns validation; Slice 7 provides deployment UI</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Save/Load</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Slice 4</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Slice 4 only</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Slice 6 owns eligibility+transaction; Slice 7 shows candidates</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Tavern/Upgrades</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Slice 6 owns functions; Slice 7 shows UI</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Guild</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Slice 6 owns progression; Slice 7 shows status</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Blacksmith</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Slice 6 owns transactions; Slice 7 shows items/costs/confirm</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Skill/Doctrine/Augment mgmt</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Slice 6 owns workflow; Slice 7 shows selection UI</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Quests/Dispatch/Explore</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Slice 6</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Slice 7</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Slice 6 owns logic; Slice 7 shows quest board</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>GIT CHECKPOINT EXPECTATIONS</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Every completed slice, every compatibility addition, and every high-risk change gets a named Git commit.</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Format: feat(scope): description OR fix(scope): description</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
dev buttons, slice 8 documentation
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Build_Plan.xlsx
+++ b/docs/CTRBLXAI_Build_Plan.xlsx
@@ -9057,7 +9057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9066,28 +9066,14 @@
           <t>SLICE MODULE OWNERSHIP AND INTEGRATION POLICY</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>FOUR MODULE CLASSIFICATIONS</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9110,7 +9096,6 @@
           <t>Later Slice Rules</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9133,7 +9118,6 @@
           <t>Consume through public APIs only</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9156,7 +9140,6 @@
           <t>No rewrite for convenience, style, cleanup, refactoring</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9179,7 +9162,6 @@
           <t>No unrelated cleanup. Ownership does not transfer.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9202,25 +9184,14 @@
           <t>Presentation must not change gameplay values</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>MODULE OWNERSHIP TABLE</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -10221,23 +10192,13 @@
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-    </row>
+    <row r="48"/>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
           <t>PROTECTED COMPLETED BEHAVIOR</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -10245,10 +10206,6 @@
           <t>After a slice is completed, its behavior is frozen. Later slices must not:</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -10256,10 +10213,6 @@
           <t>- Rewrite internals for convenience, style, or cleanup</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -10267,10 +10220,6 @@
           <t>- Create duplicate formula implementations</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -10278,10 +10227,6 @@
           <t>- Create parallel state caches</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -10289,10 +10234,6 @@
           <t>- Infer authoritative values from visual events</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -10300,28 +10241,14 @@
           <t>Backward-compatible additions may be approved via the compatibility process.</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr"/>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
           <t>DEPENDENCY DIRECTION</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -10329,10 +10256,6 @@
           <t>Authoritative rules/content → gameplay services → shared events/payloads → functional controllers → presentation views</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -10340,28 +10263,14 @@
           <t>Forbidden: combat→UI, map gen→visual layout, save→UI state, targeting→highlight appearance, formulas→presentation assets</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr"/>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="60"/>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
           <t>MIXED-SCRIPT POLICY</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -10379,8 +10288,6 @@
           <t>Rule</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -10398,8 +10305,6 @@
           <t>Mixed responsibility (rendering + input + state). Future prompts must not use as general location for new logic.</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -10417,8 +10322,6 @@
           <t>Mixed responsibility (orchestration + AI + hooks). Modifications need exact purpose + smallest diff.</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -10436,8 +10339,6 @@
           <t>Multiple slices consume. Additions need approval; no removal of existing events.</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -10455,26 +10356,14 @@
           <t>Structural only. Do not add arbitrary paths.</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr"/>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="67"/>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
           <t>OUT-OF-BATTLE OWNERSHIP</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -10497,7 +10386,6 @@
           <t>Rule</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -10517,10 +10405,9 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Slice 4 owns transactions; Slice 7 displays and emits intent</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr"/>
+          <t>Slice 4 owns transactions and data contracts; Slice 7 displays and emits intent. Slice 4 must not create visual design systems.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -10543,7 +10430,6 @@
           <t>Slice 4 owns validation; Slice 7 provides deployment UI</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -10566,7 +10452,6 @@
           <t>Slice 4 only</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -10589,7 +10474,6 @@
           <t>Slice 6 owns eligibility+transaction; Slice 7 shows candidates</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -10612,7 +10496,6 @@
           <t>Slice 6 owns functions; Slice 7 shows UI</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10635,7 +10518,6 @@
           <t>Slice 6 owns progression; Slice 7 shows status</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -10658,7 +10540,6 @@
           <t>Slice 6 owns transactions; Slice 7 shows items/costs/confirm</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -10681,7 +10562,6 @@
           <t>Slice 6 owns workflow; Slice 7 shows selection UI</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -10704,25 +10584,14 @@
           <t>Slice 6 owns logic; Slice 7 shows quest board</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr"/>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr"/>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="79"/>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
           <t>GIT CHECKPOINT EXPECTATIONS</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -10730,10 +10599,6 @@
           <t>Every completed slice, every compatibility addition, and every high-risk change gets a named Git commit.</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -10741,10 +10606,41 @@
           <t>Format: feat(scope): description OR fix(scope): description</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>SLICE 4 / SLICE 7 BOUNDARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Slice 4 owns: functional behavior, data contracts, server validation, persistence, intent/response events</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Slice 7 owns: layout, theme, colors, typography, icons, rarity borders, card appearance, responsive reflow, animations, VFX, audio, missing-asset fallbacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>If Slice 7 view does not exist: Slice 4 completes functional contract, records Slice 7 dependency, does NOT build replacement presentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>BattleVisualClient.client.lua must not become location of new menu layout, styling, or transaction authority.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>